<commit_message>
pruebas perfil cv html
</commit_message>
<xml_diff>
--- a/00soportes/Tiempos.xlsx
+++ b/00soportes/Tiempos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\cvpetrix2022\00soportes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\bazop\projects\cvpetrix2022\00soportes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ED65A2C-EA95-41D4-B4BC-24B0D2C2F01A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02532B14-35D0-4CAC-B19F-955123D31312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tiempos" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1157" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="251">
   <si>
     <t>Fecha</t>
   </si>
@@ -795,6 +795,12 @@
   <si>
     <t>Power BI</t>
   </si>
+  <si>
+    <t>TypeScript</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
 </sst>
 </file>
 
@@ -806,12 +812,19 @@
     <numFmt numFmtId="166" formatCode="_-* #,##0\ _€_-;\-* #,##0\ _€_-;_-* &quot;-&quot;\ _€_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -887,6 +900,14 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1030,36 +1051,36 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="46" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1067,12 +1088,12 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1083,19 +1104,21 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hipervínculo" xfId="2" builtinId="8"/>
@@ -1195,8 +1218,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="A1:S859" totalsRowShown="0">
-  <autoFilter ref="A1:S859" xr:uid="{00000000-0009-0000-0100-000002000000}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla2" displayName="Tabla2" ref="A1:S867" totalsRowShown="0">
+  <autoFilter ref="A1:S867" xr:uid="{00000000-0009-0000-0100-000002000000}">
     <filterColumn colId="18">
       <filters>
         <filter val="2025"/>
@@ -1233,10 +1256,10 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla1" displayName="Tabla1" ref="A1:B48" totalsRowShown="0">
-  <autoFilter ref="A1:B48" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B48">
-    <sortCondition ref="A1:A48"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla1" displayName="Tabla1" ref="A1:B49" totalsRowShown="0">
+  <autoFilter ref="A1:B49" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B49">
+    <sortCondition ref="A1:A49"/>
   </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Tecnologías"/>
@@ -1506,7 +1529,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y859"/>
+  <dimension ref="A1:Y867"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -1582,15 +1605,15 @@
       </c>
       <c r="V1" s="32">
         <f>Resumen!I2</f>
-        <v>8.6956521739130432E-2</v>
+        <v>1.4444444444444444</v>
       </c>
       <c r="W1" s="33">
         <f>Resumen!D11</f>
-        <v>9.1324200913242006E-4</v>
+        <v>2.6118721461187214E-2</v>
       </c>
       <c r="X1" s="34">
         <f>Resumen!D7+Resumen!F10</f>
-        <v>46023</v>
+        <v>46033</v>
       </c>
     </row>
     <row r="2" spans="1:24" hidden="1">
@@ -33759,7 +33782,7 @@
         <v>59</v>
       </c>
       <c r="C857" s="29">
-        <f>SUM(D857:R857)</f>
+        <f t="shared" ref="C857:C862" si="21">SUM(D857:R857)</f>
         <v>38</v>
       </c>
       <c r="D857" s="30">
@@ -33798,7 +33821,7 @@
         <v>59</v>
       </c>
       <c r="C858" s="29">
-        <f>SUM(D858:R858)</f>
+        <f t="shared" si="21"/>
         <v>82</v>
       </c>
       <c r="D858" s="30">
@@ -33839,7 +33862,7 @@
         <v>248</v>
       </c>
       <c r="C859" s="29">
-        <f>SUM(D859:R859)</f>
+        <f t="shared" si="21"/>
         <v>10</v>
       </c>
       <c r="D859" s="30">
@@ -33860,6 +33883,313 @@
       <c r="Q859" s="30"/>
       <c r="R859" s="30"/>
       <c r="S859" s="28">
+        <f>YEAR(Tabla2[[#This Row],[Fecha]])</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="860" spans="1:23">
+      <c r="A860" s="27">
+        <v>46172</v>
+      </c>
+      <c r="B860" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="C860" s="29">
+        <f t="shared" si="21"/>
+        <v>49</v>
+      </c>
+      <c r="D860" s="30">
+        <v>49</v>
+      </c>
+      <c r="E860" s="30"/>
+      <c r="F860" s="30"/>
+      <c r="G860" s="30"/>
+      <c r="H860" s="30"/>
+      <c r="I860" s="30"/>
+      <c r="J860" s="30"/>
+      <c r="K860" s="30"/>
+      <c r="L860" s="30"/>
+      <c r="M860" s="30"/>
+      <c r="N860" s="30"/>
+      <c r="O860" s="30"/>
+      <c r="P860" s="30"/>
+      <c r="Q860" s="30"/>
+      <c r="R860" s="30"/>
+      <c r="S860" s="28">
+        <f>YEAR(Tabla2[[#This Row],[Fecha]])</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="861" spans="1:23">
+      <c r="A861" s="27">
+        <v>46173</v>
+      </c>
+      <c r="B861" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="C861" s="29">
+        <f t="shared" si="21"/>
+        <v>84</v>
+      </c>
+      <c r="D861" s="30">
+        <v>4</v>
+      </c>
+      <c r="E861" s="30">
+        <v>7</v>
+      </c>
+      <c r="F861" s="30">
+        <v>7</v>
+      </c>
+      <c r="G861" s="30">
+        <v>12</v>
+      </c>
+      <c r="H861" s="30">
+        <f>60+43-49</f>
+        <v>54</v>
+      </c>
+      <c r="I861" s="30"/>
+      <c r="J861" s="30"/>
+      <c r="K861" s="30"/>
+      <c r="L861" s="30"/>
+      <c r="M861" s="30"/>
+      <c r="N861" s="30"/>
+      <c r="O861" s="30"/>
+      <c r="P861" s="30"/>
+      <c r="Q861" s="30"/>
+      <c r="R861" s="30"/>
+      <c r="S861" s="28">
+        <f>YEAR(Tabla2[[#This Row],[Fecha]])</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="862" spans="1:23">
+      <c r="A862" s="27">
+        <v>46174</v>
+      </c>
+      <c r="B862" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="C862" s="29">
+        <f t="shared" si="21"/>
+        <v>63</v>
+      </c>
+      <c r="D862" s="30">
+        <v>8</v>
+      </c>
+      <c r="E862" s="30">
+        <v>3</v>
+      </c>
+      <c r="F862" s="30">
+        <v>2</v>
+      </c>
+      <c r="G862" s="30">
+        <v>8</v>
+      </c>
+      <c r="H862" s="30">
+        <v>8</v>
+      </c>
+      <c r="I862" s="30">
+        <v>8</v>
+      </c>
+      <c r="J862" s="30">
+        <v>9</v>
+      </c>
+      <c r="K862" s="30">
+        <v>4</v>
+      </c>
+      <c r="L862" s="30">
+        <v>5</v>
+      </c>
+      <c r="M862" s="30">
+        <v>6</v>
+      </c>
+      <c r="N862" s="30">
+        <v>2</v>
+      </c>
+      <c r="O862" s="30"/>
+      <c r="P862" s="30"/>
+      <c r="Q862" s="30"/>
+      <c r="R862" s="30"/>
+      <c r="S862" s="28">
+        <f>YEAR(Tabla2[[#This Row],[Fecha]])</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="863" spans="1:23">
+      <c r="A863" s="27">
+        <v>46175</v>
+      </c>
+      <c r="B863" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="C863" s="29">
+        <f>SUM(D863:R863)</f>
+        <v>11</v>
+      </c>
+      <c r="D863" s="30">
+        <v>11</v>
+      </c>
+      <c r="E863" s="30"/>
+      <c r="F863" s="30"/>
+      <c r="G863" s="30"/>
+      <c r="H863" s="30"/>
+      <c r="I863" s="30"/>
+      <c r="J863" s="30"/>
+      <c r="K863" s="30"/>
+      <c r="L863" s="30"/>
+      <c r="M863" s="30"/>
+      <c r="N863" s="30"/>
+      <c r="O863" s="30"/>
+      <c r="P863" s="30"/>
+      <c r="Q863" s="30"/>
+      <c r="R863" s="30"/>
+      <c r="S863" s="28">
+        <f>YEAR(Tabla2[[#This Row],[Fecha]])</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="864" spans="1:23">
+      <c r="A864" s="27">
+        <v>46176</v>
+      </c>
+      <c r="B864" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="C864" s="29">
+        <f>SUM(D864:R864)</f>
+        <v>30</v>
+      </c>
+      <c r="D864" s="30">
+        <v>9</v>
+      </c>
+      <c r="E864" s="30">
+        <v>5</v>
+      </c>
+      <c r="F864" s="30">
+        <v>8</v>
+      </c>
+      <c r="G864" s="30">
+        <v>8</v>
+      </c>
+      <c r="H864" s="30"/>
+      <c r="I864" s="30"/>
+      <c r="J864" s="30"/>
+      <c r="K864" s="30"/>
+      <c r="L864" s="30"/>
+      <c r="M864" s="30"/>
+      <c r="N864" s="30"/>
+      <c r="O864" s="30"/>
+      <c r="P864" s="30"/>
+      <c r="Q864" s="30"/>
+      <c r="R864" s="30"/>
+      <c r="S864" s="28">
+        <f>YEAR(Tabla2[[#This Row],[Fecha]])</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="865" spans="1:19">
+      <c r="A865" s="27">
+        <v>46188</v>
+      </c>
+      <c r="B865" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="C865" s="29">
+        <f>SUM(D865:R865)</f>
+        <v>21</v>
+      </c>
+      <c r="D865" s="30">
+        <v>5</v>
+      </c>
+      <c r="E865" s="30">
+        <v>14</v>
+      </c>
+      <c r="F865" s="30">
+        <v>2</v>
+      </c>
+      <c r="G865" s="30"/>
+      <c r="H865" s="30"/>
+      <c r="I865" s="30"/>
+      <c r="J865" s="30"/>
+      <c r="K865" s="30"/>
+      <c r="L865" s="30"/>
+      <c r="M865" s="30"/>
+      <c r="N865" s="30"/>
+      <c r="O865" s="30"/>
+      <c r="P865" s="30"/>
+      <c r="Q865" s="30"/>
+      <c r="R865" s="30"/>
+      <c r="S865" s="28">
+        <f>YEAR(Tabla2[[#This Row],[Fecha]])</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="866" spans="1:19">
+      <c r="A866" s="27">
+        <v>46192</v>
+      </c>
+      <c r="B866" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="C866" s="29">
+        <f>SUM(D866:R866)</f>
+        <v>4</v>
+      </c>
+      <c r="D866" s="30">
+        <v>2</v>
+      </c>
+      <c r="E866" s="30">
+        <v>2</v>
+      </c>
+      <c r="F866" s="30"/>
+      <c r="G866" s="30"/>
+      <c r="H866" s="30"/>
+      <c r="I866" s="30"/>
+      <c r="J866" s="30"/>
+      <c r="K866" s="30"/>
+      <c r="L866" s="30"/>
+      <c r="M866" s="30"/>
+      <c r="N866" s="30"/>
+      <c r="O866" s="30"/>
+      <c r="P866" s="30"/>
+      <c r="Q866" s="30"/>
+      <c r="R866" s="30"/>
+      <c r="S866" s="28">
+        <f>YEAR(Tabla2[[#This Row],[Fecha]])</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="867" spans="1:19">
+      <c r="A867" s="27">
+        <v>46220</v>
+      </c>
+      <c r="B867" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="C867" s="29">
+        <f>SUM(D867:R867)</f>
+        <v>14</v>
+      </c>
+      <c r="D867" s="30">
+        <v>7</v>
+      </c>
+      <c r="E867" s="30">
+        <v>7</v>
+      </c>
+      <c r="F867" s="30"/>
+      <c r="G867" s="30"/>
+      <c r="H867" s="30"/>
+      <c r="I867" s="30"/>
+      <c r="J867" s="30"/>
+      <c r="K867" s="30"/>
+      <c r="L867" s="30"/>
+      <c r="M867" s="30"/>
+      <c r="N867" s="30"/>
+      <c r="O867" s="30"/>
+      <c r="P867" s="30"/>
+      <c r="Q867" s="30"/>
+      <c r="R867" s="30"/>
+      <c r="S867" s="28">
         <f>YEAR(Tabla2[[#This Row],[Fecha]])</f>
         <v>2026</v>
       </c>
@@ -34215,7 +34545,7 @@
       </c>
       <c r="B2" s="25">
         <f>SUM(Tabla2[Total])/(B4-B3+1)</f>
-        <v>41.46384154767388</v>
+        <v>40.059449866903286</v>
       </c>
       <c r="C2" s="25">
         <f>SUMIF(Tiempos!$S:$S,C1,Tiempos!$C:$C)/(C4-C3+1)</f>
@@ -34239,11 +34569,11 @@
       </c>
       <c r="H2" s="25">
         <f>SUMIF(Tiempos!$S:$S,H1,Tiempos!$C:$C)/(H4-H3+1)</f>
-        <v>22.633333333333333</v>
+        <v>19.296625222024868</v>
       </c>
       <c r="I2" s="25">
         <f>SUMIF(Tiempos!$S:$S,I1,Tiempos!$C:$C)/(I4-I3+1)</f>
-        <v>8.6956521739130432E-2</v>
+        <v>1.4444444444444444</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -34282,7 +34612,7 @@
       </c>
       <c r="B4" s="26">
         <f>MAX(Tabla2[Fecha])</f>
-        <v>46137</v>
+        <v>46220</v>
       </c>
       <c r="C4" s="26">
         <v>44196</v>
@@ -34301,11 +34631,11 @@
       </c>
       <c r="H4" s="26">
         <f>MAX(Tabla2[Fecha])</f>
-        <v>46137</v>
+        <v>46220</v>
       </c>
       <c r="I4" s="26">
         <f>MAX(Tabla2[Fecha])</f>
-        <v>46137</v>
+        <v>46220</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -34345,11 +34675,11 @@
       </c>
       <c r="D10" s="41">
         <f>(I4-I3+1)*I2</f>
-        <v>10</v>
+        <v>286</v>
       </c>
       <c r="F10">
         <f>ROUND(D10*F9/D9,0)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -34358,7 +34688,7 @@
       </c>
       <c r="D11" s="19">
         <f>D10/D9</f>
-        <v>9.1324200913242006E-4</v>
+        <v>2.6118721461187214E-2</v>
       </c>
     </row>
   </sheetData>
@@ -34369,14 +34699,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="15.33203125" customWidth="1"/>
     <col min="2" max="2" width="9.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:4">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -34384,7 +34714,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>61</v>
       </c>
@@ -34392,8 +34722,11 @@
         <f>SUMIF(Tiempos!B:B,A2,Tiempos!C:C)/60</f>
         <v>2.9666666666666668</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
+      <c r="D2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -34401,8 +34734,11 @@
         <f>SUMIF(Tiempos!B:B,A3,Tiempos!C:C)/60</f>
         <v>17.083333333333332</v>
       </c>
-    </row>
-    <row r="4" spans="1:2">
+      <c r="D3" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -34410,8 +34746,11 @@
         <f>SUMIF(Tiempos!B:B,A4,Tiempos!C:C)/60</f>
         <v>26.133333333333333</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
+      <c r="D4" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -34419,8 +34758,11 @@
         <f>SUMIF(Tiempos!B:B,A5,Tiempos!C:C)/60</f>
         <v>3.8</v>
       </c>
-    </row>
-    <row r="6" spans="1:2">
+      <c r="D5" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -34428,8 +34770,11 @@
         <f>SUMIF(Tiempos!B:B,A6,Tiempos!C:C)/60</f>
         <v>8.4833333333333325</v>
       </c>
-    </row>
-    <row r="7" spans="1:2">
+      <c r="D6" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -34437,8 +34782,11 @@
         <f>SUMIF(Tiempos!B:B,A7,Tiempos!C:C)/60</f>
         <v>18.466666666666665</v>
       </c>
-    </row>
-    <row r="8" spans="1:2">
+      <c r="D7" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -34446,8 +34794,11 @@
         <f>SUMIF(Tiempos!B:B,A8,Tiempos!C:C)/60</f>
         <v>1.6</v>
       </c>
-    </row>
-    <row r="9" spans="1:2">
+      <c r="D8" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>64</v>
       </c>
@@ -34455,8 +34806,11 @@
         <f>SUMIF(Tiempos!B:B,A9,Tiempos!C:C)/60</f>
         <v>1.1833333333333333</v>
       </c>
-    </row>
-    <row r="10" spans="1:2">
+      <c r="D9" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>56</v>
       </c>
@@ -34464,8 +34818,11 @@
         <f>SUMIF(Tiempos!B:B,A10,Tiempos!C:C)/60</f>
         <v>13.9</v>
       </c>
-    </row>
-    <row r="11" spans="1:2">
+      <c r="D10" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>63</v>
       </c>
@@ -34473,8 +34830,11 @@
         <f>SUMIF(Tiempos!B:B,A11,Tiempos!C:C)/60</f>
         <v>5.85</v>
       </c>
-    </row>
-    <row r="12" spans="1:2">
+      <c r="D11" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
         <v>44</v>
       </c>
@@ -34482,8 +34842,11 @@
         <f>SUMIF(Tiempos!B:B,A12,Tiempos!C:C)/60</f>
         <v>6.333333333333333</v>
       </c>
-    </row>
-    <row r="13" spans="1:2">
+      <c r="D12" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>57</v>
       </c>
@@ -34491,8 +34854,11 @@
         <f>SUMIF(Tiempos!B:B,A13,Tiempos!C:C)/60</f>
         <v>0.16666666666666666</v>
       </c>
-    </row>
-    <row r="14" spans="1:2">
+      <c r="D13" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -34500,8 +34866,11 @@
         <f>SUMIF(Tiempos!B:B,A14,Tiempos!C:C)/60</f>
         <v>54.06666666666667</v>
       </c>
-    </row>
-    <row r="15" spans="1:2">
+      <c r="D14" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15" t="s">
         <v>41</v>
       </c>
@@ -34509,8 +34878,11 @@
         <f>SUMIF(Tiempos!B:B,A15,Tiempos!C:C)/60</f>
         <v>34.283333333333331</v>
       </c>
-    </row>
-    <row r="16" spans="1:2">
+      <c r="D15" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>39</v>
       </c>
@@ -34518,17 +34890,23 @@
         <f>SUMIF(Tiempos!B:B,A16,Tiempos!C:C)/60</f>
         <v>8.5</v>
       </c>
-    </row>
-    <row r="17" spans="1:2">
+      <c r="D16" s="43" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
       <c r="A17" t="s">
         <v>22</v>
       </c>
       <c r="B17" s="22">
         <f>SUMIF(Tiempos!B:B,A17,Tiempos!C:C)/60</f>
-        <v>317.96666666666664</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
+        <v>318.03333333333336</v>
+      </c>
+      <c r="D17" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -34536,8 +34914,11 @@
         <f>SUMIF(Tiempos!B:B,A18,Tiempos!C:C)/60</f>
         <v>18.583333333333332</v>
       </c>
-    </row>
-    <row r="19" spans="1:2">
+      <c r="D18" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19" t="s">
         <v>30</v>
       </c>
@@ -34545,8 +34926,11 @@
         <f>SUMIF(Tiempos!B:B,A19,Tiempos!C:C)/60</f>
         <v>1.8833333333333333</v>
       </c>
-    </row>
-    <row r="20" spans="1:2">
+      <c r="D19" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -34554,8 +34938,11 @@
         <f>SUMIF(Tiempos!B:B,A20,Tiempos!C:C)/60</f>
         <v>37.049999999999997</v>
       </c>
-    </row>
-    <row r="21" spans="1:2">
+      <c r="D20" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" t="s">
         <v>58</v>
       </c>
@@ -34563,8 +34950,11 @@
         <f>SUMIF(Tiempos!B:B,A21,Tiempos!C:C)/60</f>
         <v>6.3166666666666664</v>
       </c>
-    </row>
-    <row r="22" spans="1:2">
+      <c r="D21" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -34572,8 +34962,11 @@
         <f>SUMIF(Tiempos!B:B,A22,Tiempos!C:C)/60</f>
         <v>52.15</v>
       </c>
-    </row>
-    <row r="23" spans="1:2">
+      <c r="D22" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23" t="s">
         <v>19</v>
       </c>
@@ -34581,8 +34974,11 @@
         <f>SUMIF(Tiempos!B:B,A23,Tiempos!C:C)/60</f>
         <v>109.75</v>
       </c>
-    </row>
-    <row r="24" spans="1:2">
+      <c r="D23" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -34590,8 +34986,11 @@
         <f>SUMIF(Tiempos!B:B,A24,Tiempos!C:C)/60</f>
         <v>26.516666666666666</v>
       </c>
-    </row>
-    <row r="25" spans="1:2">
+      <c r="D24" s="43" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -34599,8 +34998,11 @@
         <f>SUMIF(Tiempos!B:B,A25,Tiempos!C:C)/60</f>
         <v>91</v>
       </c>
-    </row>
-    <row r="26" spans="1:2">
+      <c r="D25" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
       <c r="A26" t="s">
         <v>51</v>
       </c>
@@ -34608,8 +35010,11 @@
         <f>SUMIF(Tiempos!B:B,A26,Tiempos!C:C)/60</f>
         <v>2.15</v>
       </c>
-    </row>
-    <row r="27" spans="1:2">
+      <c r="D26" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -34617,8 +35022,11 @@
         <f>SUMIF(Tiempos!B:B,A27,Tiempos!C:C)/60</f>
         <v>250.13333333333333</v>
       </c>
-    </row>
-    <row r="28" spans="1:2">
+      <c r="D27" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
       <c r="A28" t="s">
         <v>24</v>
       </c>
@@ -34626,8 +35034,11 @@
         <f>SUMIF(Tiempos!B:B,A28,Tiempos!C:C)/60</f>
         <v>47.4</v>
       </c>
-    </row>
-    <row r="29" spans="1:2">
+      <c r="D28" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -34635,8 +35046,11 @@
         <f>SUMIF(Tiempos!B:B,A29,Tiempos!C:C)/60</f>
         <v>2.9333333333333331</v>
       </c>
-    </row>
-    <row r="30" spans="1:2">
+      <c r="D29" s="43" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -34644,8 +35058,11 @@
         <f>SUMIF(Tiempos!B:B,A30,Tiempos!C:C)/60</f>
         <v>40</v>
       </c>
-    </row>
-    <row r="31" spans="1:2">
+      <c r="D30" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
       <c r="A31" t="s">
         <v>60</v>
       </c>
@@ -34653,8 +35070,11 @@
         <f>SUMIF(Tiempos!B:B,A31,Tiempos!C:C)/60</f>
         <v>5.0999999999999996</v>
       </c>
-    </row>
-    <row r="32" spans="1:2">
+      <c r="D31" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
       <c r="A32" t="s">
         <v>28</v>
       </c>
@@ -34662,8 +35082,11 @@
         <f>SUMIF(Tiempos!B:B,A32,Tiempos!C:C)/60</f>
         <v>45.9</v>
       </c>
-    </row>
-    <row r="33" spans="1:2">
+      <c r="D32" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
       <c r="A33" t="s">
         <v>43</v>
       </c>
@@ -34671,8 +35094,11 @@
         <f>SUMIF(Tiempos!B:B,A33,Tiempos!C:C)/60</f>
         <v>9.0166666666666675</v>
       </c>
-    </row>
-    <row r="34" spans="1:2">
+      <c r="D33" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
       <c r="A34" t="s">
         <v>50</v>
       </c>
@@ -34680,8 +35106,11 @@
         <f>SUMIF(Tiempos!B:B,A34,Tiempos!C:C)/60</f>
         <v>13.25</v>
       </c>
-    </row>
-    <row r="35" spans="1:2">
+      <c r="D34" s="42" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
       <c r="A35" t="s">
         <v>52</v>
       </c>
@@ -34689,8 +35118,11 @@
         <f>SUMIF(Tiempos!B:B,A35,Tiempos!C:C)/60</f>
         <v>3.35</v>
       </c>
-    </row>
-    <row r="36" spans="1:2">
+      <c r="D35" s="43" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
       <c r="A36" t="s">
         <v>248</v>
       </c>
@@ -34698,8 +35130,11 @@
         <f>SUMIF(Tiempos!B:B,A36,Tiempos!C:C)/60</f>
         <v>0.16666666666666666</v>
       </c>
-    </row>
-    <row r="37" spans="1:2">
+      <c r="D36" s="43" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
       <c r="A37" t="s">
         <v>53</v>
       </c>
@@ -34707,8 +35142,11 @@
         <f>SUMIF(Tiempos!B:B,A37,Tiempos!C:C)/60</f>
         <v>17.25</v>
       </c>
-    </row>
-    <row r="38" spans="1:2">
+      <c r="D37" s="43" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
       <c r="A38" t="s">
         <v>36</v>
       </c>
@@ -34716,8 +35154,11 @@
         <f>SUMIF(Tiempos!B:B,A38,Tiempos!C:C)/60</f>
         <v>21.083333333333332</v>
       </c>
-    </row>
-    <row r="39" spans="1:2">
+      <c r="D38" s="43" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
       <c r="A39" t="s">
         <v>34</v>
       </c>
@@ -34725,8 +35166,11 @@
         <f>SUMIF(Tiempos!B:B,A39,Tiempos!C:C)/60</f>
         <v>51.016666666666666</v>
       </c>
-    </row>
-    <row r="40" spans="1:2">
+      <c r="D39" s="43" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
       <c r="A40" t="s">
         <v>46</v>
       </c>
@@ -34734,8 +35178,11 @@
         <f>SUMIF(Tiempos!B:B,A40,Tiempos!C:C)/60</f>
         <v>0.6166666666666667</v>
       </c>
-    </row>
-    <row r="41" spans="1:2">
+      <c r="D40" s="43" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
       <c r="A41" t="s">
         <v>32</v>
       </c>
@@ -34743,8 +35190,11 @@
         <f>SUMIF(Tiempos!B:B,A41,Tiempos!C:C)/60</f>
         <v>3.2166666666666668</v>
       </c>
-    </row>
-    <row r="42" spans="1:2">
+      <c r="D41" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
       <c r="A42" t="s">
         <v>49</v>
       </c>
@@ -34753,7 +35203,7 @@
         <v>1.9333333333333333</v>
       </c>
     </row>
-    <row r="43" spans="1:2">
+    <row r="43" spans="1:4">
       <c r="A43" t="s">
         <v>29</v>
       </c>
@@ -34761,8 +35211,11 @@
         <f>SUMIF(Tiempos!B:B,A43,Tiempos!C:C)/60</f>
         <v>7.8666666666666663</v>
       </c>
-    </row>
-    <row r="44" spans="1:2">
+      <c r="D43" s="43" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
       <c r="A44" t="s">
         <v>59</v>
       </c>
@@ -34770,41 +35223,65 @@
         <f>SUMIF(Tiempos!B:B,A44,Tiempos!C:C)/60</f>
         <v>16.333333333333332</v>
       </c>
-    </row>
-    <row r="45" spans="1:2">
+      <c r="D44" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>33</v>
+        <v>249</v>
       </c>
       <c r="B45" s="22">
         <f>SUMIF(Tiempos!B:B,A45,Tiempos!C:C)/60</f>
-        <v>89.85</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2">
+        <v>4.5333333333333332</v>
+      </c>
+      <c r="D45" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="B46" s="22">
         <f>SUMIF(Tiempos!B:B,A46,Tiempos!C:C)/60</f>
-        <v>5.8166666666666664</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2">
+        <v>89.85</v>
+      </c>
+      <c r="D46" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="B47" s="22">
         <f>SUMIF(Tiempos!B:B,A47,Tiempos!C:C)/60</f>
-        <v>0.41666666666666669</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2">
+        <v>5.8166666666666664</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B48" s="22">
         <f>SUMIF(Tiempos!B:B,A48,Tiempos!C:C)/60</f>
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D48" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49" s="22">
+        <f>SUMIF(Tiempos!B:B,A49,Tiempos!C:C)/60</f>
         <v>1.4666666666666666</v>
+      </c>
+      <c r="D49" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -34812,8 +35289,9 @@
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>